<commit_message>
Started working functions in the Excel Practice TAB 1 like production level
</commit_message>
<xml_diff>
--- a/Excel_Workbook.xlsx
+++ b/Excel_Workbook.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Excel Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6442F1EE-E2DC-4B5E-83EC-1090BDC5A898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9033073-67A5-4524-B664-6102ACBEB4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{430F5E05-F8E5-4D72-914A-86006FE066F8}"/>
   </bookViews>
@@ -874,6 +874,13 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -883,15 +890,8 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1239,37 +1239,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" ht="21.6" thickBot="1">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="E1" s="17" t="s">
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="E1" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="R1" s="18" t="s">
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="R1" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="S1" s="18"/>
-      <c r="T1" s="18"/>
-      <c r="U1" s="18"/>
-      <c r="V1" s="18"/>
+      <c r="S1" s="21"/>
+      <c r="T1" s="21"/>
+      <c r="U1" s="21"/>
+      <c r="V1" s="21"/>
       <c r="W1" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="X1" s="18" t="s">
+      <c r="X1" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="Y1" s="18"/>
-      <c r="Z1" s="18"/>
-      <c r="AA1" s="19"/>
-      <c r="AB1" s="19"/>
+      <c r="Y1" s="21"/>
+      <c r="Z1" s="21"/>
+      <c r="AA1" s="22"/>
+      <c r="AB1" s="22"/>
     </row>
     <row r="2" spans="1:32" ht="16.8" thickTop="1" thickBot="1">
       <c r="A2" s="1" t="s">
@@ -1356,10 +1356,10 @@
       <c r="AD2" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="AE2" s="21" t="s">
+      <c r="AE2" s="17" t="s">
         <v>197</v>
       </c>
-      <c r="AF2" s="21" t="s">
+      <c r="AF2" s="17" t="s">
         <v>198</v>
       </c>
     </row>
@@ -1465,8 +1465,8 @@
         <f>REPLACE(N3,7,17,"BBBBBB")</f>
         <v>souravBBBBBB</v>
       </c>
-      <c r="AE3" s="20" t="str">
-        <f>IFERROR(LEFT(N3,FIND("@",SUBSTITUTE(N3," ","@",2))-1),N3)</f>
+      <c r="AE3" s="16" t="str">
+        <f>LEFT(N3,LEN(N3)-LEN(TRIM(RIGHT(SUBSTITUTE(N3," ",REPT(" ",100)),100)))-1)</f>
         <v>sourav joshi</v>
       </c>
       <c r="AF3" s="3" t="str">
@@ -1576,7 +1576,7 @@
         <f t="shared" ref="AD4:AD67" si="12">REPLACE(N4,7,17,"BBBBBB")</f>
         <v>TriggeBBBBBB</v>
       </c>
-      <c r="AE4" s="20" t="str">
+      <c r="AE4" s="16" t="str">
         <f t="shared" ref="AE4:AE67" si="13">IFERROR(LEFT(N4,FIND("@",SUBSTITUTE(N4," ","@",2))-1),N4)</f>
         <v>Triggered Insaan</v>
       </c>
@@ -1687,7 +1687,7 @@
         <f t="shared" si="12"/>
         <v>SONY MBBBBBB</v>
       </c>
-      <c r="AE5" s="20" t="str">
+      <c r="AE5" s="16" t="str">
         <f t="shared" si="13"/>
         <v>SONY MUSIC</v>
       </c>
@@ -1798,7 +1798,7 @@
         <f t="shared" si="12"/>
         <v>Sony MBBBBBB</v>
       </c>
-      <c r="AE6" s="20" t="str">
+      <c r="AE6" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Sony Music</v>
       </c>
@@ -1909,7 +1909,7 @@
         <f t="shared" si="12"/>
         <v>souravBBBBBB</v>
       </c>
-      <c r="AE7" s="20" t="str">
+      <c r="AE7" s="16" t="str">
         <f t="shared" si="13"/>
         <v>sourav joshi</v>
       </c>
@@ -2020,7 +2020,7 @@
         <f t="shared" si="12"/>
         <v>Zee MuBBBBBB</v>
       </c>
-      <c r="AE8" s="20" t="str">
+      <c r="AE8" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Zee Music</v>
       </c>
@@ -2131,7 +2131,7 @@
         <f t="shared" si="12"/>
         <v>factteBBBBBB</v>
       </c>
-      <c r="AE9" s="20" t="str">
+      <c r="AE9" s="16" t="str">
         <f t="shared" si="13"/>
         <v xml:space="preserve">facttechz </v>
       </c>
@@ -2242,7 +2242,7 @@
         <f t="shared" si="12"/>
         <v>T-serIBBBBBB</v>
       </c>
-      <c r="AE10" s="20" t="str">
+      <c r="AE10" s="16" t="str">
         <f t="shared" si="13"/>
         <v>T-serIES</v>
       </c>
@@ -2353,7 +2353,7 @@
         <f t="shared" si="12"/>
         <v>T-serIBBBBBB</v>
       </c>
-      <c r="AE11" s="20" t="str">
+      <c r="AE11" s="16" t="str">
         <f t="shared" si="13"/>
         <v>T-serIES</v>
       </c>
@@ -2464,7 +2464,7 @@
         <f t="shared" si="12"/>
         <v>TechniBBBBBB</v>
       </c>
-      <c r="AE12" s="20" t="str">
+      <c r="AE12" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Technical Guruji</v>
       </c>
@@ -2575,7 +2575,7 @@
         <f t="shared" si="12"/>
         <v xml:space="preserve"> SET IBBBBBB</v>
       </c>
-      <c r="AE13" s="20" t="str">
+      <c r="AE13" s="16" t="str">
         <f t="shared" si="13"/>
         <v xml:space="preserve"> SET</v>
       </c>
@@ -2686,7 +2686,7 @@
         <f t="shared" si="12"/>
         <v>kids DBBBBBB</v>
       </c>
-      <c r="AE14" s="20" t="str">
+      <c r="AE14" s="16" t="str">
         <f t="shared" si="13"/>
         <v>kids Diana</v>
       </c>
@@ -2797,7 +2797,7 @@
         <f t="shared" si="12"/>
         <v>t-seriBBBBBB</v>
       </c>
-      <c r="AE15" s="20" t="str">
+      <c r="AE15" s="16" t="str">
         <f t="shared" si="13"/>
         <v xml:space="preserve">t-series </v>
       </c>
@@ -2908,7 +2908,7 @@
         <f t="shared" si="12"/>
         <v>MySmarBBBBBB</v>
       </c>
-      <c r="AE16" s="20" t="str">
+      <c r="AE16" s="16" t="str">
         <f t="shared" si="13"/>
         <v>MySmartPrice</v>
       </c>
@@ -3019,7 +3019,7 @@
         <f t="shared" si="12"/>
         <v>Canal BBBBBB</v>
       </c>
-      <c r="AE17" s="20" t="str">
+      <c r="AE17" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Canal Kondzilla</v>
       </c>
@@ -3130,7 +3130,7 @@
         <f t="shared" si="12"/>
         <v xml:space="preserve"> SET IBBBBBB</v>
       </c>
-      <c r="AE18" s="20" t="str">
+      <c r="AE18" s="16" t="str">
         <f t="shared" si="13"/>
         <v xml:space="preserve"> SET</v>
       </c>
@@ -3232,7 +3232,7 @@
         <f t="shared" si="12"/>
         <v>bb ki BBBBBB</v>
       </c>
-      <c r="AE19" s="20" t="str">
+      <c r="AE19" s="16" t="str">
         <f t="shared" si="13"/>
         <v>bb ki</v>
       </c>
@@ -3334,7 +3334,7 @@
         <f t="shared" si="12"/>
         <v>badabuBBBBBB</v>
       </c>
-      <c r="AE20" s="20" t="str">
+      <c r="AE20" s="16" t="str">
         <f t="shared" si="13"/>
         <v xml:space="preserve">badabun </v>
       </c>
@@ -3436,7 +3436,7 @@
         <f t="shared" si="12"/>
         <v>SONY MBBBBBB</v>
       </c>
-      <c r="AE21" s="20" t="str">
+      <c r="AE21" s="16" t="str">
         <f t="shared" si="13"/>
         <v>SONY MUSIC</v>
       </c>
@@ -3538,7 +3538,7 @@
         <f t="shared" si="12"/>
         <v>TechniBBBBBB</v>
       </c>
-      <c r="AE22" s="20" t="str">
+      <c r="AE22" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Technical Guruji</v>
       </c>
@@ -3640,7 +3640,7 @@
         <f t="shared" si="12"/>
         <v>FACTTEBBBBBB</v>
       </c>
-      <c r="AE23" s="20" t="str">
+      <c r="AE23" s="16" t="str">
         <f t="shared" si="13"/>
         <v>FACTTECHZ</v>
       </c>
@@ -3742,7 +3742,7 @@
         <f t="shared" si="12"/>
         <v>Sony MBBBBBB</v>
       </c>
-      <c r="AE24" s="20" t="str">
+      <c r="AE24" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Sony Music</v>
       </c>
@@ -3844,7 +3844,7 @@
         <f t="shared" si="12"/>
         <v>TechniBBBBBB</v>
       </c>
-      <c r="AE25" s="20" t="str">
+      <c r="AE25" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Technical Guruji</v>
       </c>
@@ -3946,7 +3946,7 @@
         <f t="shared" si="12"/>
         <v>Aaj TaBBBBBB</v>
       </c>
-      <c r="AE26" s="20" t="str">
+      <c r="AE26" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Aaj Tak</v>
       </c>
@@ -4048,7 +4048,7 @@
         <f t="shared" si="12"/>
         <v>MySmarBBBBBB</v>
       </c>
-      <c r="AE27" s="20" t="str">
+      <c r="AE27" s="16" t="str">
         <f t="shared" si="13"/>
         <v>MySmartPrice</v>
       </c>
@@ -4150,7 +4150,7 @@
         <f t="shared" si="12"/>
         <v>VanossBBBBBB</v>
       </c>
-      <c r="AE28" s="20" t="str">
+      <c r="AE28" s="16" t="str">
         <f t="shared" si="13"/>
         <v>VanossGaming</v>
       </c>
@@ -4252,7 +4252,7 @@
         <f t="shared" si="12"/>
         <v>coComeBBBBBBmes</v>
       </c>
-      <c r="AE29" s="20" t="str">
+      <c r="AE29" s="16" t="str">
         <f t="shared" si="13"/>
         <v>coComelon -</v>
       </c>
@@ -4354,7 +4354,7 @@
         <f t="shared" si="12"/>
         <v>Total BBBBBB</v>
       </c>
-      <c r="AE30" s="20" t="str">
+      <c r="AE30" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Total Gaming</v>
       </c>
@@ -4456,7 +4456,7 @@
         <f t="shared" si="12"/>
         <v>Dude PBBBBBB</v>
       </c>
-      <c r="AE31" s="20" t="str">
+      <c r="AE31" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Dude Perfect</v>
       </c>
@@ -4558,7 +4558,7 @@
         <f t="shared" si="12"/>
         <v>MarkipBBBBBB</v>
       </c>
-      <c r="AE32" s="20" t="str">
+      <c r="AE32" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Markiplier</v>
       </c>
@@ -4637,7 +4637,7 @@
         <f t="shared" si="12"/>
         <v>Tech BBBBBBB</v>
       </c>
-      <c r="AE33" s="20" t="str">
+      <c r="AE33" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Tech Burner</v>
       </c>
@@ -4716,7 +4716,7 @@
         <f t="shared" si="12"/>
         <v>kids dBBBBBB</v>
       </c>
-      <c r="AE34" s="20" t="str">
+      <c r="AE34" s="16" t="str">
         <f t="shared" si="13"/>
         <v>kids diana</v>
       </c>
@@ -4795,7 +4795,7 @@
         <f t="shared" si="12"/>
         <v>sony mBBBBBB</v>
       </c>
-      <c r="AE35" s="20" t="str">
+      <c r="AE35" s="16" t="str">
         <f t="shared" si="13"/>
         <v>sony music</v>
       </c>
@@ -4874,7 +4874,7 @@
         <f t="shared" si="12"/>
         <v>Round2BBBBBB</v>
       </c>
-      <c r="AE36" s="20" t="str">
+      <c r="AE36" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Round2hell</v>
       </c>
@@ -4953,7 +4953,7 @@
         <f t="shared" si="12"/>
         <v xml:space="preserve"> SET IBBBBBB</v>
       </c>
-      <c r="AE37" s="20" t="str">
+      <c r="AE37" s="16" t="str">
         <f t="shared" si="13"/>
         <v xml:space="preserve"> SET</v>
       </c>
@@ -5032,7 +5032,7 @@
         <f t="shared" si="12"/>
         <v>vanossBBBBBB</v>
       </c>
-      <c r="AE38" s="20" t="str">
+      <c r="AE38" s="16" t="str">
         <f t="shared" si="13"/>
         <v xml:space="preserve">vanossgaming </v>
       </c>
@@ -5111,7 +5111,7 @@
         <f t="shared" si="12"/>
         <v xml:space="preserve"> SET IBBBBBB</v>
       </c>
-      <c r="AE39" s="20" t="str">
+      <c r="AE39" s="16" t="str">
         <f t="shared" si="13"/>
         <v xml:space="preserve"> SET</v>
       </c>
@@ -5190,7 +5190,7 @@
         <f t="shared" si="12"/>
         <v>coComeBBBBBBmes</v>
       </c>
-      <c r="AE40" s="20" t="str">
+      <c r="AE40" s="16" t="str">
         <f t="shared" si="13"/>
         <v>coComelon -</v>
       </c>
@@ -5269,7 +5269,7 @@
         <f t="shared" si="12"/>
         <v>BB Ki BBBBBB</v>
       </c>
-      <c r="AE41" s="20" t="str">
+      <c r="AE41" s="16" t="str">
         <f t="shared" si="13"/>
         <v>BB Ki</v>
       </c>
@@ -5348,7 +5348,7 @@
         <f t="shared" si="12"/>
         <v>PEWdieBBBBBB</v>
       </c>
-      <c r="AE42" s="20" t="str">
+      <c r="AE42" s="16" t="str">
         <f t="shared" si="13"/>
         <v>PEWdiePie</v>
       </c>
@@ -5427,7 +5427,7 @@
         <f t="shared" si="12"/>
         <v>COCOMEBBBBBBMES</v>
       </c>
-      <c r="AE43" s="20" t="str">
+      <c r="AE43" s="16" t="str">
         <f t="shared" si="13"/>
         <v>COCOMELON -</v>
       </c>
@@ -5506,7 +5506,7 @@
         <f t="shared" si="12"/>
         <v>Tech BBBBBBB</v>
       </c>
-      <c r="AE44" s="20" t="str">
+      <c r="AE44" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Tech Burner</v>
       </c>
@@ -5585,7 +5585,7 @@
         <f t="shared" si="12"/>
         <v>PEWDIEBBBBBB</v>
       </c>
-      <c r="AE45" s="20" t="str">
+      <c r="AE45" s="16" t="str">
         <f t="shared" si="13"/>
         <v>PEWDIEPIE</v>
       </c>
@@ -5664,7 +5664,7 @@
         <f t="shared" si="12"/>
         <v>MarkipBBBBBB</v>
       </c>
-      <c r="AE46" s="20" t="str">
+      <c r="AE46" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Markiplier</v>
       </c>
@@ -5743,7 +5743,7 @@
         <f t="shared" si="12"/>
         <v>Desi GBBBBBB</v>
       </c>
-      <c r="AE47" s="20" t="str">
+      <c r="AE47" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Desi Gamers</v>
       </c>
@@ -5822,7 +5822,7 @@
         <f t="shared" si="12"/>
         <v>VANOSSBBBBBB</v>
       </c>
-      <c r="AE48" s="20" t="str">
+      <c r="AE48" s="16" t="str">
         <f t="shared" si="13"/>
         <v>VANOSSGAMING</v>
       </c>
@@ -5901,7 +5901,7 @@
         <f t="shared" si="12"/>
         <v>Tech BBBBBBB</v>
       </c>
-      <c r="AE49" s="20" t="str">
+      <c r="AE49" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Tech Burner</v>
       </c>
@@ -5980,7 +5980,7 @@
         <f t="shared" si="12"/>
         <v>PEWdieBBBBBB</v>
       </c>
-      <c r="AE50" s="20" t="str">
+      <c r="AE50" s="16" t="str">
         <f t="shared" si="13"/>
         <v>PEWdiePie</v>
       </c>
@@ -6059,7 +6059,7 @@
         <f t="shared" si="12"/>
         <v>5-MINUBBBBBB</v>
       </c>
-      <c r="AE51" s="20" t="str">
+      <c r="AE51" s="16" t="str">
         <f t="shared" si="13"/>
         <v>5-MINUTE CRAFTS</v>
       </c>
@@ -6138,7 +6138,7 @@
         <f t="shared" si="12"/>
         <v>MySmarBBBBBB</v>
       </c>
-      <c r="AE52" s="20" t="str">
+      <c r="AE52" s="16" t="str">
         <f t="shared" si="13"/>
         <v>MySmartPrice</v>
       </c>
@@ -6217,7 +6217,7 @@
         <f t="shared" si="12"/>
         <v>PEWdieBBBBBB</v>
       </c>
-      <c r="AE53" s="20" t="str">
+      <c r="AE53" s="16" t="str">
         <f t="shared" si="13"/>
         <v>PEWdiePie</v>
       </c>
@@ -6296,7 +6296,7 @@
         <f t="shared" si="12"/>
         <v>coComeBBBBBBmes</v>
       </c>
-      <c r="AE54" s="20" t="str">
+      <c r="AE54" s="16" t="str">
         <f t="shared" si="13"/>
         <v>coComelon -</v>
       </c>
@@ -6375,7 +6375,7 @@
         <f t="shared" si="12"/>
         <v>Sony MBBBBBB</v>
       </c>
-      <c r="AE55" s="20" t="str">
+      <c r="AE55" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Sony Music</v>
       </c>
@@ -6454,7 +6454,7 @@
         <f t="shared" si="12"/>
         <v>VanossBBBBBB</v>
       </c>
-      <c r="AE56" s="20" t="str">
+      <c r="AE56" s="16" t="str">
         <f t="shared" si="13"/>
         <v>VanossGaming</v>
       </c>
@@ -6533,7 +6533,7 @@
         <f t="shared" si="12"/>
         <v>TriggeBBBBBB</v>
       </c>
-      <c r="AE57" s="20" t="str">
+      <c r="AE57" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Triggered Insaan</v>
       </c>
@@ -6612,7 +6612,7 @@
         <f t="shared" si="12"/>
         <v>BadabuBBBBBB</v>
       </c>
-      <c r="AE58" s="20" t="str">
+      <c r="AE58" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Badabun</v>
       </c>
@@ -6691,7 +6691,7 @@
         <f t="shared" si="12"/>
         <v>round2BBBBBB</v>
       </c>
-      <c r="AE59" s="20" t="str">
+      <c r="AE59" s="16" t="str">
         <f t="shared" si="13"/>
         <v>round2hell</v>
       </c>
@@ -6770,7 +6770,7 @@
         <f t="shared" si="12"/>
         <v>KIDS DBBBBBB</v>
       </c>
-      <c r="AE60" s="20" t="str">
+      <c r="AE60" s="16" t="str">
         <f t="shared" si="13"/>
         <v>KIDS DIANA</v>
       </c>
@@ -6849,7 +6849,7 @@
         <f t="shared" si="12"/>
         <v>canal BBBBBB</v>
       </c>
-      <c r="AE61" s="20" t="str">
+      <c r="AE61" s="16" t="str">
         <f t="shared" si="13"/>
         <v>canal kondzilla</v>
       </c>
@@ -6928,7 +6928,7 @@
         <f t="shared" si="12"/>
         <v>desi gBBBBBB</v>
       </c>
-      <c r="AE62" s="20" t="str">
+      <c r="AE62" s="16" t="str">
         <f t="shared" si="13"/>
         <v>desi gamers</v>
       </c>
@@ -7007,7 +7007,7 @@
         <f t="shared" si="12"/>
         <v>ASHISHBBBBBB</v>
       </c>
-      <c r="AE63" s="20" t="str">
+      <c r="AE63" s="16" t="str">
         <f t="shared" si="13"/>
         <v>ASHISH CHANCHLANI</v>
       </c>
@@ -7086,7 +7086,7 @@
         <f t="shared" si="12"/>
         <v>mysmarBBBBBB</v>
       </c>
-      <c r="AE64" s="20" t="str">
+      <c r="AE64" s="16" t="str">
         <f t="shared" si="13"/>
         <v>mysmartprice</v>
       </c>
@@ -7165,7 +7165,7 @@
         <f t="shared" si="12"/>
         <v>ZEE MUBBBBBB</v>
       </c>
-      <c r="AE65" s="20" t="str">
+      <c r="AE65" s="16" t="str">
         <f t="shared" si="13"/>
         <v>ZEE MUSIC</v>
       </c>
@@ -7244,7 +7244,7 @@
         <f t="shared" si="12"/>
         <v>Desi GBBBBBB</v>
       </c>
-      <c r="AE66" s="20" t="str">
+      <c r="AE66" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Desi Gamers</v>
       </c>
@@ -7323,7 +7323,7 @@
         <f t="shared" si="12"/>
         <v>Total BBBBBB</v>
       </c>
-      <c r="AE67" s="20" t="str">
+      <c r="AE67" s="16" t="str">
         <f t="shared" si="13"/>
         <v>Total Gaming</v>
       </c>
@@ -7402,7 +7402,7 @@
         <f t="shared" ref="AD68:AD102" si="27">REPLACE(N68,7,17,"BBBBBB")</f>
         <v>AshishBBBBBB</v>
       </c>
-      <c r="AE68" s="20" t="str">
+      <c r="AE68" s="16" t="str">
         <f t="shared" ref="AE68:AE102" si="28">IFERROR(LEFT(N68,FIND("@",SUBSTITUTE(N68," ","@",2))-1),N68)</f>
         <v>Ashish Chanchlani</v>
       </c>
@@ -7481,7 +7481,7 @@
         <f t="shared" si="27"/>
         <v xml:space="preserve">ashishBBBBBB  </v>
       </c>
-      <c r="AE69" s="20" t="str">
+      <c r="AE69" s="16" t="str">
         <f t="shared" si="28"/>
         <v>ashish chanchlani</v>
       </c>
@@ -7560,7 +7560,7 @@
         <f t="shared" si="27"/>
         <v>total BBBBBB</v>
       </c>
-      <c r="AE70" s="20" t="str">
+      <c r="AE70" s="16" t="str">
         <f t="shared" si="28"/>
         <v>total gaming</v>
       </c>
@@ -7639,7 +7639,7 @@
         <f t="shared" si="27"/>
         <v>MARKIPBBBBBB</v>
       </c>
-      <c r="AE71" s="20" t="str">
+      <c r="AE71" s="16" t="str">
         <f t="shared" si="28"/>
         <v>MARKIPLIER</v>
       </c>
@@ -7718,7 +7718,7 @@
         <f t="shared" si="27"/>
         <v>Nas DaBBBBBB</v>
       </c>
-      <c r="AE72" s="20" t="str">
+      <c r="AE72" s="16" t="str">
         <f t="shared" si="28"/>
         <v>Nas Daily</v>
       </c>
@@ -7797,7 +7797,7 @@
         <f t="shared" si="27"/>
         <v>Sony MBBBBBB</v>
       </c>
-      <c r="AE73" s="20" t="str">
+      <c r="AE73" s="16" t="str">
         <f t="shared" si="28"/>
         <v>Sony Music</v>
       </c>
@@ -7876,7 +7876,7 @@
         <f t="shared" si="27"/>
         <v>carrymBBBBBB</v>
       </c>
-      <c r="AE74" s="20" t="str">
+      <c r="AE74" s="16" t="str">
         <f t="shared" si="28"/>
         <v>carryminati</v>
       </c>
@@ -7955,7 +7955,7 @@
         <f t="shared" si="27"/>
         <v>yrfBBBBBB</v>
       </c>
-      <c r="AE75" s="20" t="str">
+      <c r="AE75" s="16" t="str">
         <f t="shared" si="28"/>
         <v>yrf</v>
       </c>
@@ -8034,7 +8034,7 @@
         <f t="shared" si="27"/>
         <v>tech bBBBBBB</v>
       </c>
-      <c r="AE76" s="20" t="str">
+      <c r="AE76" s="16" t="str">
         <f t="shared" si="28"/>
         <v>tech burner</v>
       </c>
@@ -8113,7 +8113,7 @@
         <f t="shared" si="27"/>
         <v>MrBeasBBBBBB</v>
       </c>
-      <c r="AE77" s="20" t="str">
+      <c r="AE77" s="16" t="str">
         <f t="shared" si="28"/>
         <v xml:space="preserve">MrBeast </v>
       </c>
@@ -8192,7 +8192,7 @@
         <f t="shared" si="27"/>
         <v>TRIGGEBBBBBB</v>
       </c>
-      <c r="AE78" s="20" t="str">
+      <c r="AE78" s="16" t="str">
         <f t="shared" si="28"/>
         <v>TRIGGERED INSAAN</v>
       </c>
@@ -8271,7 +8271,7 @@
         <f t="shared" si="27"/>
         <v>kids DBBBBBB</v>
       </c>
-      <c r="AE79" s="20" t="str">
+      <c r="AE79" s="16" t="str">
         <f t="shared" si="28"/>
         <v>kids Diana</v>
       </c>
@@ -8350,7 +8350,7 @@
         <f t="shared" si="27"/>
         <v>ROUND2BBBBBB</v>
       </c>
-      <c r="AE80" s="20" t="str">
+      <c r="AE80" s="16" t="str">
         <f t="shared" si="28"/>
         <v>ROUND2HELL</v>
       </c>
@@ -8429,7 +8429,7 @@
         <f t="shared" si="27"/>
         <v>Round2BBBBBB</v>
       </c>
-      <c r="AE81" s="20" t="str">
+      <c r="AE81" s="16" t="str">
         <f t="shared" si="28"/>
         <v>Round2hell</v>
       </c>
@@ -8508,7 +8508,7 @@
         <f t="shared" si="27"/>
         <v>FactTeBBBBBB</v>
       </c>
-      <c r="AE82" s="20" t="str">
+      <c r="AE82" s="16" t="str">
         <f t="shared" si="28"/>
         <v>FactTechz</v>
       </c>
@@ -8587,7 +8587,7 @@
         <f t="shared" si="27"/>
         <v>TechniBBBBBB</v>
       </c>
-      <c r="AE83" s="20" t="str">
+      <c r="AE83" s="16" t="str">
         <f t="shared" si="28"/>
         <v>Technical Guruji</v>
       </c>
@@ -8666,7 +8666,7 @@
         <f t="shared" si="27"/>
         <v>TRIGGEBBBBBB</v>
       </c>
-      <c r="AE84" s="20" t="str">
+      <c r="AE84" s="16" t="str">
         <f t="shared" si="28"/>
         <v>TRIGGERED INSAAN</v>
       </c>
@@ -8745,7 +8745,7 @@
         <f t="shared" si="27"/>
         <v>mrbeasBBBBBB</v>
       </c>
-      <c r="AE85" s="20" t="str">
+      <c r="AE85" s="16" t="str">
         <f t="shared" si="28"/>
         <v>mrbeast</v>
       </c>
@@ -8824,7 +8824,7 @@
         <f t="shared" si="27"/>
         <v>YRFBBBBBB</v>
       </c>
-      <c r="AE86" s="20" t="str">
+      <c r="AE86" s="16" t="str">
         <f t="shared" si="28"/>
         <v>YRF</v>
       </c>
@@ -8903,7 +8903,7 @@
         <f t="shared" si="27"/>
         <v>TRIGGEBBBBBB</v>
       </c>
-      <c r="AE87" s="20" t="str">
+      <c r="AE87" s="16" t="str">
         <f t="shared" si="28"/>
         <v>TRIGGERED INSAAN</v>
       </c>
@@ -8982,7 +8982,7 @@
         <f t="shared" si="27"/>
         <v>bb ki BBBBBB</v>
       </c>
-      <c r="AE88" s="20" t="str">
+      <c r="AE88" s="16" t="str">
         <f t="shared" si="28"/>
         <v>bb ki</v>
       </c>
@@ -9061,7 +9061,7 @@
         <f t="shared" si="27"/>
         <v>VanossBBBBBB</v>
       </c>
-      <c r="AE89" s="20" t="str">
+      <c r="AE89" s="16" t="str">
         <f t="shared" si="28"/>
         <v>VanossGaming</v>
       </c>
@@ -9140,7 +9140,7 @@
         <f t="shared" si="27"/>
         <v>PEWDIEBBBBBB</v>
       </c>
-      <c r="AE90" s="20" t="str">
+      <c r="AE90" s="16" t="str">
         <f t="shared" si="28"/>
         <v>PEWDIEPIE</v>
       </c>
@@ -9219,7 +9219,7 @@
         <f t="shared" si="27"/>
         <v>MySmarBBBBBB</v>
       </c>
-      <c r="AE91" s="20" t="str">
+      <c r="AE91" s="16" t="str">
         <f t="shared" si="28"/>
         <v>MySmartPrice</v>
       </c>
@@ -9298,7 +9298,7 @@
         <f t="shared" si="27"/>
         <v>coComeBBBBBBmes</v>
       </c>
-      <c r="AE92" s="20" t="str">
+      <c r="AE92" s="16" t="str">
         <f t="shared" si="28"/>
         <v>coComelon -</v>
       </c>
@@ -9377,7 +9377,7 @@
         <f t="shared" si="27"/>
         <v>KIDS DBBBBBB</v>
       </c>
-      <c r="AE93" s="20" t="str">
+      <c r="AE93" s="16" t="str">
         <f t="shared" si="28"/>
         <v>KIDS DIANA</v>
       </c>
@@ -9456,7 +9456,7 @@
         <f t="shared" si="27"/>
         <v>VanossBBBBBB</v>
       </c>
-      <c r="AE94" s="20" t="str">
+      <c r="AE94" s="16" t="str">
         <f t="shared" si="28"/>
         <v>VanossGaming</v>
       </c>
@@ -9535,7 +9535,7 @@
         <f t="shared" si="27"/>
         <v>MarkipBBBBBB</v>
       </c>
-      <c r="AE95" s="20" t="str">
+      <c r="AE95" s="16" t="str">
         <f t="shared" si="28"/>
         <v>Markiplier</v>
       </c>
@@ -9614,7 +9614,7 @@
         <f t="shared" si="27"/>
         <v>Round2BBBBBB</v>
       </c>
-      <c r="AE96" s="20" t="str">
+      <c r="AE96" s="16" t="str">
         <f t="shared" si="28"/>
         <v xml:space="preserve">Round2hell </v>
       </c>
@@ -9693,7 +9693,7 @@
         <f t="shared" si="27"/>
         <v>ZEE MUBBBBBB</v>
       </c>
-      <c r="AE97" s="20" t="str">
+      <c r="AE97" s="16" t="str">
         <f t="shared" si="28"/>
         <v>ZEE MUSIC</v>
       </c>
@@ -9772,7 +9772,7 @@
         <f t="shared" si="27"/>
         <v>MrBeasBBBBBB</v>
       </c>
-      <c r="AE98" s="20" t="str">
+      <c r="AE98" s="16" t="str">
         <f t="shared" si="28"/>
         <v xml:space="preserve">MrBeast </v>
       </c>
@@ -9851,7 +9851,7 @@
         <f t="shared" si="27"/>
         <v>CANAL BBBBBB</v>
       </c>
-      <c r="AE99" s="20" t="str">
+      <c r="AE99" s="16" t="str">
         <f t="shared" si="28"/>
         <v>CANAL KONDZILLA</v>
       </c>
@@ -9930,7 +9930,7 @@
         <f t="shared" si="27"/>
         <v>TriggeBBBBBB</v>
       </c>
-      <c r="AE100" s="20" t="str">
+      <c r="AE100" s="16" t="str">
         <f t="shared" si="28"/>
         <v>Triggered Insaan</v>
       </c>
@@ -10009,7 +10009,7 @@
         <f t="shared" si="27"/>
         <v>TechniBBBBBB</v>
       </c>
-      <c r="AE101" s="20" t="str">
+      <c r="AE101" s="16" t="str">
         <f t="shared" si="28"/>
         <v>Technical Guruji</v>
       </c>
@@ -10088,7 +10088,7 @@
         <f t="shared" si="27"/>
         <v>MySmarBBBBBB</v>
       </c>
-      <c r="AE102" s="20" t="str">
+      <c r="AE102" s="16" t="str">
         <f t="shared" si="28"/>
         <v>MySmartPrice</v>
       </c>
@@ -10108,23 +10108,23 @@
     <row r="105" spans="5:32" ht="15.6">
       <c r="E105" s="9"/>
       <c r="I105" s="10"/>
-      <c r="M105" s="22" t="s">
+      <c r="M105" s="18" t="s">
         <v>199</v>
       </c>
-      <c r="N105" s="22"/>
-      <c r="O105" s="22"/>
-      <c r="P105" s="22"/>
-      <c r="Q105" s="22"/>
-      <c r="R105" s="22"/>
-      <c r="S105" s="22"/>
-      <c r="T105" s="22"/>
-      <c r="U105" s="22"/>
-      <c r="V105" s="22"/>
-      <c r="W105" s="22"/>
-      <c r="X105" s="22"/>
-      <c r="Y105" s="22"/>
-      <c r="Z105" s="22"/>
-      <c r="AA105" s="22"/>
+      <c r="N105" s="18"/>
+      <c r="O105" s="18"/>
+      <c r="P105" s="18"/>
+      <c r="Q105" s="18"/>
+      <c r="R105" s="18"/>
+      <c r="S105" s="18"/>
+      <c r="T105" s="18"/>
+      <c r="U105" s="18"/>
+      <c r="V105" s="18"/>
+      <c r="W105" s="18"/>
+      <c r="X105" s="18"/>
+      <c r="Y105" s="18"/>
+      <c r="Z105" s="18"/>
+      <c r="AA105" s="18"/>
     </row>
     <row r="106" spans="5:32">
       <c r="E106" s="9"/>

</xml_diff>

<commit_message>
Tried to change the formula for the first and lastname but didnt change it finally
</commit_message>
<xml_diff>
--- a/Excel_Workbook.xlsx
+++ b/Excel_Workbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\Excel Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9033073-67A5-4524-B664-6102ACBEB4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EE24B80-3730-4F72-BC31-133B54D2B4D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{430F5E05-F8E5-4D72-914A-86006FE066F8}"/>
   </bookViews>
@@ -1466,7 +1466,7 @@
         <v>souravBBBBBB</v>
       </c>
       <c r="AE3" s="16" t="str">
-        <f>LEFT(N3,LEN(N3)-LEN(TRIM(RIGHT(SUBSTITUTE(N3," ",REPT(" ",100)),100)))-1)</f>
+        <f>IFERROR(LEFT(N3,FIND("@",SUBSTITUTE(N3," ","@",2))-1),N3)</f>
         <v>sourav joshi</v>
       </c>
       <c r="AF3" s="3" t="str">
@@ -1577,7 +1577,7 @@
         <v>TriggeBBBBBB</v>
       </c>
       <c r="AE4" s="16" t="str">
-        <f t="shared" ref="AE4:AE67" si="13">IFERROR(LEFT(N4,FIND("@",SUBSTITUTE(N4," ","@",2))-1),N4)</f>
+        <f t="shared" ref="AE3:AE67" si="13">IFERROR(LEFT(N4,FIND("@",SUBSTITUTE(N4," ","@",2))-1),N4)</f>
         <v>Triggered Insaan</v>
       </c>
       <c r="AF4" s="3" t="str">

</xml_diff>